<commit_message>
updated research detail and cleaned up temporary csv files during conversion int /data folder
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -3127,7 +3127,7 @@
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   This writes lps/lp-import.csv preserving existing Considered=yes rows.</t>
+          <t xml:space="preserve">   This writes data/lp-import.csv preserving existing Considered=yes rows.</t>
         </is>
       </c>
     </row>
@@ -3168,7 +3168,7 @@
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>6. .venv/bin/python scripts/convert.py export   →  output.xlsx (pipeline view)</t>
+          <t>6. .venv/bin/python scripts/convert.py export   →  output.xlsx (from data/output.csv)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
partial research update and input.xlsx and output.xlsx visual upgrades and tweaks
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -11,7 +11,7 @@
     <sheet name="How to use" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$L$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,11 +49,11 @@
       <color rgb="009C0006"/>
     </font>
     <font>
-      <color rgb="00AAAAAA"/>
+      <color rgb="00000000"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00AAAAAA"/>
+      <color rgb="00000000"/>
     </font>
     <font>
       <b val="1"/>
@@ -64,9 +64,6 @@
       <sz val="11"/>
     </font>
     <font/>
-    <font>
-      <color rgb="00444444"/>
-    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -179,7 +176,7 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -545,74 +542,80 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K46"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Country</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Website</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>First Name</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Last Name</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Email address</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Considered</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Stage</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Score /100</t>
         </is>
@@ -621,2462 +624,2593 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Pension Fund</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
           <t>VBV-Pensionskasse AG</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Austria</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>https://www.vbv.at</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Andreas</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Zakostelsky</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>General Director</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>a.zakostelsky@vbv.at</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>drafted</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>90/100</t>
-        </is>
+      <c r="L2" s="4" t="n">
+        <v>92</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Pension Fund</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
           <t>Valida Pensionskasse AG</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Austria</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>https://www.valida.at</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Martin</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Sardelic</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Martin.sardelic@valida.at</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>linkedin.com/in/martin-sardelic-75b36126</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J3" s="6" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>70/100</t>
-        </is>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L3" s="6" t="n">
+        <v>68</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Pension Fund</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
           <t>APK Pensionskasse AG</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Austria</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>https://www.apk-pensionskasse.at</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Beate</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Wolf</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Chairwoman of the Directory</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>beate.wolf@apk.at</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>linkedin.com/in/beate-wolf-06581b96</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>78/100</t>
-        </is>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>82</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Pension Fund</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
           <t>Bonus Pensionskasse AG</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Austria</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>https://www.bonuspensionskasse.at</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Michael</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Scherhammer</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Chairman (CEO)</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>michael.scherhammer@bonusvorsorge.at</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>88/100</t>
-        </is>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="n">
+        <v>88</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Pension Fund</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
           <t>Allianz Pensionskasse AG</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Austria</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>https://www.allianz.at</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Andreas</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Csurda</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Chairman (CEO)</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>andreas.csurda@allianz.at</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>78/100</t>
-        </is>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>78</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Pension Fund</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
           <t>Raiffeisen Pensionskasse AG</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Austria</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>https://www.raiffeisen-pk.at</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Martin</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Sardelic</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Martin.sardelic@valida.at</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr"/>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J7" s="7" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>30/100</t>
-        </is>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L7" s="7" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Vorsorgekasse</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
           <t>VBV Vorsorgekasse AG</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Austria</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>https://www.vorsorgekasse.at</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>Andreas</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Zakostelsky</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>General Director</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>a.zakostelsky@vbv.at</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J8" s="6" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>55/100</t>
-        </is>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L8" s="6" t="n">
+        <v>58</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Corporate Pension</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
           <t>IBM Pensionskasse AG</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>Austria</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>https://www.ibm.com/us-en</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>Gerald</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>Leberbauer</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr">
+      <c r="G9" s="8" t="inlineStr">
         <is>
           <t>CFO</t>
         </is>
       </c>
-      <c r="G9" s="8" t="inlineStr">
+      <c r="H9" s="8" t="inlineStr">
         <is>
           <t>gerald.leberbauer@ibm.com</t>
         </is>
       </c>
-      <c r="H9" s="8" t="inlineStr"/>
-      <c r="I9" s="9" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J9" s="10" t="inlineStr">
+      <c r="I9" s="8" t="inlineStr"/>
+      <c r="J9" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
         <is>
           <t>skip</t>
         </is>
       </c>
-      <c r="K9" s="8" t="inlineStr">
-        <is>
-          <t>5/100</t>
-        </is>
+      <c r="L9" s="10" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Pension Fund</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
           <t>Bundespensionskasse AG</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Austria</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>https://bundespensionskasse.at/</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Marcus</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Klug</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>CFO</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>marcus.klug@bundespensionskasse.at</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>linkedin.com/in/marcusklug</t>
         </is>
       </c>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J10" s="11" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>48/100</t>
-        </is>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L10" s="11" t="n">
+        <v>48</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
+          <t>EU</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Pension Fund</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>Resaver</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>EU</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>https://www.resaver.eu/</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>Beata</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Cseresznye</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Pension Fund Manager</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>beata.cseresznye@resaver.eu</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr"/>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J11" s="7" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>25/100</t>
-        </is>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L11" s="7" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Corporate Pension</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
           <t>Nestle Pensionsfonds AG</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>Austria</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr"/>
       <c r="D12" s="8" t="inlineStr"/>
       <c r="E12" s="8" t="inlineStr"/>
       <c r="F12" s="8" t="inlineStr"/>
       <c r="G12" s="8" t="inlineStr"/>
       <c r="H12" s="8" t="inlineStr"/>
-      <c r="I12" s="9" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J12" s="10" t="inlineStr">
+      <c r="I12" s="8" t="inlineStr"/>
+      <c r="J12" s="8" t="inlineStr"/>
+      <c r="K12" s="9" t="inlineStr">
         <is>
           <t>skip</t>
         </is>
       </c>
-      <c r="K12" s="8" t="inlineStr">
-        <is>
-          <t>5/100</t>
-        </is>
+      <c r="L12" s="10" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Insurance Company</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
           <t>Donau Versicherung</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Austria</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>https://www.donauversicherung.at/</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>Wolfgang</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Petschko</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>CIO</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>w.petschko@donauversicherung.at</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>linkedin.com/in/wolfgang-petschko-12077aba</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J13" s="11" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>48/100</t>
-        </is>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L13" s="11" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Pension Fund</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
           <t>Sozialversicherungspensionskasse AG</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Austria</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>https://www.svpk.at/</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>Sascha</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>König</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>CFO</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>sascha.koenig@svpk.at</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J14" s="11" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>38/100</t>
-        </is>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L14" s="11" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Insurance Company</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
           <t>Vienna Insurance Group (VIG)</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Austria</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>https://group.vig.com</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>Hartwig</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>Löger</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>hartwig.loeger@vig.com</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr"/>
-      <c r="I15" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>78/100</t>
-        </is>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Insurance Company</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
           <t>Uniqa Insurance Group</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Austria</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>https://www.uniqa.at</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>Andreas</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Brandstatter</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>andreas.brandstatter@uniqa.at</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr"/>
-      <c r="I16" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J16" s="6" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>68/100</t>
-        </is>
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L16" s="6" t="n">
+        <v>68</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Insurance Company</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
           <t>Generali Versicherung AG</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Austria</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>https://www.generali.at</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>Gregor</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>Pilgram</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>greogor.pilgram@generali.com</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>linkedin.com/in/gregor-pilgram-6492542</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J17" s="11" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>48/100</t>
-        </is>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L17" s="11" t="n">
+        <v>48</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Insurance Company</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
           <t>Allianz Österreich</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Austria</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>https://www.allianz.at</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>Daniel</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Matic</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>daniel.matic@allianz.at</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>linkedin.com/in/daniel-matić-2478642b2</t>
         </is>
       </c>
-      <c r="I18" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J18" s="11" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>45/100</t>
-        </is>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L18" s="11" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Insurance Company</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
           <t>Grawe Group</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Austria</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>https://www.grawe.at</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>Klaus</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>Scheitegel</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>klaus.scheitegel@grawe.at</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr"/>
-      <c r="I19" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J19" s="4" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>78/100</t>
-        </is>
+      <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Insurance Company</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
           <t>Ergo Versicherung AG</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Austria</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>https://www.ergo-versicherung.at</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>Philipp</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Wassenberg</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>philipp.wassenberg@ergo-versicherung.at</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>linkedin.com/in/philipp-wassenberg-333639aa</t>
         </is>
       </c>
-      <c r="I20" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J20" s="11" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>35/100</t>
-        </is>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L20" s="11" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Insurance Company</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
           <t>Merkur Versicherung AG</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Austria</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>https://www.merkur.at</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>Christian</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>Kladiva</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>christian.kladiva@merkur.at</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>linkedin.com/in/christian-kladiva-b018b21b9</t>
         </is>
       </c>
-      <c r="I21" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J21" s="7" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr">
-        <is>
-          <t>30/100</t>
-        </is>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L21" s="7" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Insurance Company</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
           <t>Helvetia Versicherungen</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Austria</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>https://www.helvetia.at</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>Thomas</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Neusiedler</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>thomas.neusiedler@helvetia.at</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="I22" s="2" t="inlineStr">
         <is>
           <t>linkedin.com/in/thomas-neusiedler-28b65082</t>
         </is>
       </c>
-      <c r="I22" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J22" s="6" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>55/100</t>
-        </is>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L22" s="6" t="n">
+        <v>55</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Insurance Company</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
           <t>Oberösterreichische Versicherung</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Austria</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>https://www.ooev.at</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>Othmar</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>Nagl</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>o.nagl@ooev.at</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="I23" s="2" t="inlineStr">
         <is>
           <t>linkedin.com/in/othmarnagl</t>
         </is>
       </c>
-      <c r="I23" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J23" s="6" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>62/100</t>
-        </is>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L23" s="6" t="n">
+        <v>62</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Insurance Company</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
           <t>Zürich Versicherung AG</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Austria</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>https://www.zurich.at</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>Luciano</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Cirinà</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>luciano.cirina@at.zurich.com</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>linkedin.com/in/luciano-cirinà-515425158</t>
         </is>
       </c>
-      <c r="I24" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J24" s="11" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>35/100</t>
-        </is>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L24" s="11" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Insurance Company</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
           <t>Croatia osiguranje d.d.</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Croatia</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>https://www.crosig.hr</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>Davor</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t>Tomašković</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t>davor.tomaskovic@crosig.hr</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="I25" s="2" t="inlineStr">
         <is>
           <t>linkedin.com/in/davortomaskovic</t>
         </is>
       </c>
-      <c r="I25" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J25" s="11" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>40/100</t>
-        </is>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L25" s="11" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Insurance Company</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
           <t>Euroherc osiguranje</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Croatia</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>https://www.euroherc.hr</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
       <c r="G26" s="2" t="inlineStr"/>
       <c r="H26" s="2" t="inlineStr"/>
-      <c r="I26" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J26" s="7" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t>28/100</t>
-        </is>
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K26" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L26" s="7" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Insurance Company</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
           <t>Adriatic Osiguranje</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Croatia</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>https://www.adriatic-osiguranje.hr/</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>Nino</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>Pavić</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>nino.pavic@adriatic-osiguranje.hr</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr"/>
-      <c r="I27" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J27" s="7" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K27" s="2" t="inlineStr">
-        <is>
-          <t>28/100</t>
-        </is>
+      <c r="I27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L27" s="7" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Insurance Company</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
           <t>Allianz Hrvatska</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Croatia</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>https://www.allianz.hr</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>Marijana</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Jakovac</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>jakovacm@allianz.hr</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="I28" s="2" t="inlineStr">
         <is>
           <t>linkedin.com/in/marijana-jakovac-46586b1a</t>
         </is>
       </c>
-      <c r="I28" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J28" s="7" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K28" s="2" t="inlineStr">
-        <is>
-          <t>30/100</t>
-        </is>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K28" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L28" s="7" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Insurance Company</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
           <t>Wiener Osiguranje VIG</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>Croatia</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>https://www.wiener.hr</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>Tamara</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>Rendić</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>trendic@wiener.at</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="I29" s="2" t="inlineStr">
         <is>
           <t>linkedin.com/in/tamara-rendić-208a3792</t>
         </is>
       </c>
-      <c r="I29" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J29" s="11" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K29" s="2" t="inlineStr">
-        <is>
-          <t>40/100</t>
-        </is>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K29" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L29" s="11" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Insurance Company</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
           <t>Grawe Hrvatska</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>Croatia</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>https://www.grawe.hr</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>Nataša</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Kapetanović</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>natasa.kapetanovic@grawe.hr</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr">
+      <c r="I30" s="2" t="inlineStr">
         <is>
           <t>linkedin.com/in/nataša-kapetanović-710aa2116</t>
         </is>
       </c>
-      <c r="I30" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J30" s="11" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K30" s="2" t="inlineStr">
-        <is>
-          <t>45/100</t>
-        </is>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K30" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L30" s="11" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Insurance Company</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
           <t>Generali osiguranje</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Croatia</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>https://www.generali.hr</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>Mario</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>Carini</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>mario.carini@generali.hr</t>
         </is>
       </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="I31" s="2" t="inlineStr">
         <is>
           <t>linkedin.com/in/mario-carini-6030513</t>
         </is>
       </c>
-      <c r="I31" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J31" s="7" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K31" s="2" t="inlineStr">
-        <is>
-          <t>28/100</t>
-        </is>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K31" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L31" s="7" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Insurance Company</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
           <t>Triglav osiguranje</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Croatia</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>https://www.triglav.hr</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>Tedo</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Djekanović</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>Chairman of the Supervisory Board</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>tedo.djekanovic@triglav.hr</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr">
+      <c r="I32" s="2" t="inlineStr">
         <is>
           <t>linkedin.com/in/tedo-djekanovic-0691aa2b2</t>
         </is>
       </c>
-      <c r="I32" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J32" s="11" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K32" s="2" t="inlineStr">
-        <is>
-          <t>38/100</t>
-        </is>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K32" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L32" s="11" t="n">
+        <v>38</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Insurance Company</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
           <t>Merkur osiguranje</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>Croatia</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>https://www.merkur.hr</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>Marko</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>Klemenčič</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>marko.klemencic@merkur.hr</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr">
+      <c r="I33" s="2" t="inlineStr">
         <is>
           <t>linkedin.com/in/marko-klemenčič-a230757a</t>
         </is>
       </c>
-      <c r="I33" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J33" s="7" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K33" s="2" t="inlineStr">
-        <is>
-          <t>25/100</t>
-        </is>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K33" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L33" s="7" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>Mandatory Pension Fund</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
           <t>AZ Mandatory Pension Fund</t>
         </is>
       </c>
-      <c r="B34" s="8" t="inlineStr">
-        <is>
-          <t>Croatia</t>
-        </is>
-      </c>
-      <c r="C34" s="8" t="inlineStr">
+      <c r="D34" s="8" t="inlineStr">
         <is>
           <t>https://www.azfond.hr</t>
         </is>
       </c>
-      <c r="D34" s="8" t="inlineStr">
+      <c r="E34" s="8" t="inlineStr">
         <is>
           <t>Kristijan</t>
         </is>
       </c>
-      <c r="E34" s="8" t="inlineStr">
+      <c r="F34" s="8" t="inlineStr">
         <is>
           <t>Buk</t>
         </is>
       </c>
-      <c r="F34" s="8" t="inlineStr">
+      <c r="G34" s="8" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G34" s="8" t="inlineStr">
+      <c r="H34" s="8" t="inlineStr">
         <is>
           <t>kristijan.buk@azfond.hr</t>
         </is>
       </c>
-      <c r="H34" s="8" t="inlineStr"/>
-      <c r="I34" s="9" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J34" s="10" t="inlineStr">
+      <c r="I34" s="8" t="inlineStr"/>
+      <c r="J34" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K34" s="9" t="inlineStr">
         <is>
           <t>skip</t>
         </is>
       </c>
-      <c r="K34" s="8" t="inlineStr">
-        <is>
-          <t>15/100</t>
-        </is>
+      <c r="L34" s="10" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>Mandatory Pension Fund</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
           <t>ABA Mandatory Pension Fund</t>
         </is>
       </c>
-      <c r="B35" s="8" t="inlineStr">
-        <is>
-          <t>Croatia</t>
-        </is>
-      </c>
-      <c r="C35" s="8" t="inlineStr">
+      <c r="D35" s="8" t="inlineStr">
         <is>
           <t>https://www.pbz.hr</t>
         </is>
       </c>
-      <c r="D35" s="8" t="inlineStr">
+      <c r="E35" s="8" t="inlineStr">
         <is>
           <t>Dinko</t>
         </is>
       </c>
-      <c r="E35" s="8" t="inlineStr">
+      <c r="F35" s="8" t="inlineStr">
         <is>
           <t>Lucić</t>
         </is>
       </c>
-      <c r="F35" s="8" t="inlineStr">
+      <c r="G35" s="8" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G35" s="8" t="inlineStr">
+      <c r="H35" s="8" t="inlineStr">
         <is>
           <t>dinko.lucic@pbz.hr</t>
         </is>
       </c>
-      <c r="H35" s="8" t="inlineStr">
+      <c r="I35" s="8" t="inlineStr">
         <is>
           <t>linkedin.com/in/dinko-lucic-phd-aa009085</t>
         </is>
       </c>
-      <c r="I35" s="9" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J35" s="10" t="inlineStr">
+      <c r="J35" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K35" s="9" t="inlineStr">
         <is>
           <t>skip</t>
         </is>
       </c>
-      <c r="K35" s="8" t="inlineStr">
-        <is>
-          <t>15/100</t>
-        </is>
+      <c r="L35" s="10" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Voluntary Pension Fund</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
           <t>Raiffeisen Voluntary Pension Fund</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>Croatia</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>https://www.rmf.hr/</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>Gordan</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Šumanović</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>gordan.sumanovic@rmf.hr</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr">
+      <c r="I36" s="2" t="inlineStr">
         <is>
           <t>linkedin.com/in/gordan-sumanovic-cfa-1916676</t>
         </is>
       </c>
-      <c r="I36" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J36" s="7" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K36" s="2" t="inlineStr">
-        <is>
-          <t>32/100</t>
-        </is>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K36" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L36" s="7" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>Mandatory Pension Fund</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
           <t>AZ Mandatory B Category</t>
         </is>
       </c>
-      <c r="B37" s="8" t="inlineStr">
-        <is>
-          <t>Croatia</t>
-        </is>
-      </c>
-      <c r="C37" s="8" t="inlineStr">
+      <c r="D37" s="8" t="inlineStr">
         <is>
           <t>https://www.azfond.hr</t>
         </is>
       </c>
-      <c r="D37" s="8" t="inlineStr">
+      <c r="E37" s="8" t="inlineStr">
         <is>
           <t>Kristijan</t>
         </is>
       </c>
-      <c r="E37" s="8" t="inlineStr">
+      <c r="F37" s="8" t="inlineStr">
         <is>
           <t>Buk</t>
         </is>
       </c>
-      <c r="F37" s="8" t="inlineStr">
+      <c r="G37" s="8" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G37" s="8" t="inlineStr">
+      <c r="H37" s="8" t="inlineStr">
         <is>
           <t>kristijan.buk@azfond.hr</t>
         </is>
       </c>
-      <c r="H37" s="8" t="inlineStr"/>
-      <c r="I37" s="9" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J37" s="10" t="inlineStr">
+      <c r="I37" s="8" t="inlineStr"/>
+      <c r="J37" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K37" s="9" t="inlineStr">
         <is>
           <t>skip</t>
         </is>
       </c>
-      <c r="K37" s="8" t="inlineStr">
-        <is>
-          <t>15/100</t>
-        </is>
+      <c r="L37" s="10" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
         <is>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>Mandatory Pension Fund</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
           <t>Erste Mandatory Pension Fund</t>
         </is>
       </c>
-      <c r="B38" s="8" t="inlineStr">
-        <is>
-          <t>Croatia</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="inlineStr">
+      <c r="D38" s="8" t="inlineStr">
         <is>
           <t>https://www.pbz.hr</t>
         </is>
       </c>
-      <c r="D38" s="8" t="inlineStr">
+      <c r="E38" s="8" t="inlineStr">
         <is>
           <t>Petar</t>
         </is>
       </c>
-      <c r="E38" s="8" t="inlineStr">
+      <c r="F38" s="8" t="inlineStr">
         <is>
           <t>Vlaić</t>
         </is>
       </c>
-      <c r="F38" s="8" t="inlineStr">
+      <c r="G38" s="8" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G38" s="8" t="inlineStr">
+      <c r="H38" s="8" t="inlineStr">
         <is>
           <t>petar.vlaic@ersteplavi.hr</t>
         </is>
       </c>
-      <c r="H38" s="8" t="inlineStr">
+      <c r="I38" s="8" t="inlineStr">
         <is>
           <t>linkedin.com/in/petar-vlaić-cfa-02498216</t>
         </is>
       </c>
-      <c r="I38" s="9" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J38" s="7" t="inlineStr">
+      <c r="J38" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K38" s="9" t="inlineStr">
         <is>
           <t>skip</t>
         </is>
       </c>
-      <c r="K38" s="8" t="inlineStr">
-        <is>
-          <t>20/100</t>
-        </is>
+      <c r="L38" s="10" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Voluntary Pension Fund</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
           <t>AZ Voluntary Pension Fund</t>
         </is>
       </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>Croatia</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>https://www.azfond.hr</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>Kristijan</t>
         </is>
       </c>
-      <c r="E39" s="2" t="inlineStr">
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>Buk</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr">
+      <c r="G39" s="2" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G39" s="2" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>kristijan.buk@azfond.hr</t>
         </is>
       </c>
-      <c r="H39" s="2" t="inlineStr"/>
-      <c r="I39" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J39" s="7" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K39" s="2" t="inlineStr">
-        <is>
-          <t>30/100</t>
-        </is>
+      <c r="I39" s="2" t="inlineStr"/>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K39" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L39" s="7" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Voluntary Pension Fund</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
           <t>Erste Voluntary Fund</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>Croatia</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>https://www.erstebank.hr</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>Petar</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Vlaić</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>petar.vlaic@ersteplavi.hr</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr"/>
-      <c r="I40" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J40" s="7" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K40" s="2" t="inlineStr">
-        <is>
-          <t>32/100</t>
-        </is>
+      <c r="I40" s="2" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K40" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L40" s="7" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>Voluntary Pension Fund</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
           <t>Croatia osiguranje Voluntary</t>
         </is>
       </c>
-      <c r="B41" s="8" t="inlineStr">
-        <is>
-          <t>Croatia</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
+      <c r="D41" s="8" t="inlineStr">
         <is>
           <t>https://www.crosig-trecistup.hr/</t>
         </is>
       </c>
-      <c r="D41" s="8" t="inlineStr">
+      <c r="E41" s="8" t="inlineStr">
         <is>
           <t>Radojka</t>
         </is>
       </c>
-      <c r="E41" s="8" t="inlineStr">
+      <c r="F41" s="8" t="inlineStr">
         <is>
           <t>Hainski</t>
         </is>
       </c>
-      <c r="F41" s="8" t="inlineStr">
+      <c r="G41" s="8" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G41" s="8" t="inlineStr">
+      <c r="H41" s="8" t="inlineStr">
         <is>
           <t>radojka.hainski@crosig.hr</t>
         </is>
       </c>
-      <c r="H41" s="8" t="inlineStr">
+      <c r="I41" s="8" t="inlineStr">
         <is>
           <t>linkedin.com/in/radojka-hainski-frm-79289522</t>
         </is>
       </c>
-      <c r="I41" s="9" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J41" s="10" t="inlineStr">
+      <c r="J41" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K41" s="9" t="inlineStr">
         <is>
           <t>skip</t>
         </is>
       </c>
-      <c r="K41" s="8" t="inlineStr">
-        <is>
-          <t>12/100</t>
-        </is>
+      <c r="L41" s="10" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Czech Republic</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Pension Society</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
           <t>ČSOB Penzijní společnost</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Czech Republic</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>https://www.csob-penze.cz</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>Marcela</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>Suchanková</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr">
         <is>
           <t>msuchankova@csob.cz</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr">
+      <c r="I42" s="2" t="inlineStr">
         <is>
           <t>linkedin.com/in/marcela-suchankova-49b6b012</t>
         </is>
       </c>
-      <c r="I42" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J42" s="11" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K42" s="2" t="inlineStr">
-        <is>
-          <t>52/100</t>
-        </is>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K42" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L42" s="11" t="n">
+        <v>52</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
+          <t>Czech Republic</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Pension Society</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
           <t>Allianz Penzijní společnost</t>
         </is>
       </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>Czech Republic</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>https://www.allianz.cz</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="E43" s="2" t="inlineStr">
         <is>
           <t>Dušan</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="F43" s="2" t="inlineStr">
         <is>
           <t>Quis</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr">
+      <c r="G43" s="2" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G43" s="2" t="inlineStr">
+      <c r="H43" s="2" t="inlineStr">
         <is>
           <t>dusan.quis@allianz.cz</t>
         </is>
       </c>
-      <c r="H43" s="2" t="inlineStr">
+      <c r="I43" s="2" t="inlineStr">
         <is>
           <t>linkedin.com/in/dusan-quis-9625355b</t>
         </is>
       </c>
-      <c r="I43" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J43" s="11" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K43" s="2" t="inlineStr">
-        <is>
-          <t>40/100</t>
-        </is>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K43" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L43" s="11" t="n">
+        <v>42</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
+          <t>Czech Republic</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Pension Society</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
           <t>Česká spořitelna - penzijní</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>Czech Republic</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>https://www.csps.cz/cs/penzijni-sporeni</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>Aleš</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>Poklop</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr">
         <is>
           <t>ales.poklop@csps.cz</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr">
+      <c r="I44" s="2" t="inlineStr">
         <is>
           <t>linkedin.com/in/aleš-poklop-45690a255</t>
         </is>
       </c>
-      <c r="I44" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J44" s="4" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K44" s="2" t="inlineStr">
-        <is>
-          <t>78/100</t>
-        </is>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K44" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L44" s="4" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
+          <t>Czech Republic</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Pension Society</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
           <t>NN Penzijní společnost</t>
         </is>
       </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>Czech Republic</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>https://www.nn.cz</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="E45" s="2" t="inlineStr">
         <is>
           <t>Yoram</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="F45" s="2" t="inlineStr">
         <is>
           <t>Schwarz</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr">
+      <c r="G45" s="2" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G45" s="2" t="inlineStr">
+      <c r="H45" s="2" t="inlineStr">
         <is>
           <t>yoram.schwarz@nn.cz</t>
         </is>
       </c>
-      <c r="H45" s="2" t="inlineStr">
+      <c r="I45" s="2" t="inlineStr">
         <is>
           <t>linkedin.com/in/yoram-schwarz-a925021</t>
         </is>
       </c>
-      <c r="I45" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J45" s="11" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K45" s="2" t="inlineStr">
-        <is>
-          <t>50/100</t>
-        </is>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K45" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L45" s="11" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
+          <t>Czech Republic</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Pension Society</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
           <t>Generali penzijní společnost</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>Czech Republic</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>https://www.generalipenze.cz/</t>
         </is>
       </c>
-      <c r="D46" s="2" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>Jana</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>Zelinková</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr">
         <is>
           <t>jana.zelinkova@generalipenze.cz</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr">
+      <c r="I46" s="2" t="inlineStr">
         <is>
           <t>linkedin.com/in/jana-zelinkova-76920b1a6</t>
         </is>
       </c>
-      <c r="I46" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J46" s="6" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="K46" s="2" t="inlineStr">
-        <is>
-          <t>72/100</t>
-        </is>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K46" s="5" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="L46" s="6" t="n">
+        <v>72</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K1"/>
+  <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>